<commit_message>
Update Bioethanol inventory data.xlsx
</commit_message>
<xml_diff>
--- a/tutorials/FuelLCAModel/Bioethanol inventory data.xlsx
+++ b/tutorials/FuelLCAModel/Bioethanol inventory data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6a7a065f75d1a80f/Desktop/BEST502 Advanced LCA/BEST502-AdvancedLCA-Tutorials/tutorials/FuelLCAModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4D7AEAB-47B6-4DA4-8AFB-CFC6D2D40190}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{D4D7AEAB-47B6-4DA4-8AFB-CFC6D2D40190}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF4DF244-3E4A-4061-933E-D12CA7036065}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E88F3882-B473-4446-BA84-AEE73DC13D43}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E88F3882-B473-4446-BA84-AEE73DC13D43}"/>
   </bookViews>
   <sheets>
     <sheet name="Inventory data (Bioethanol)" sheetId="1" r:id="rId1"/>
@@ -137,9 +137,6 @@
     <t>CFR Data Workbook: sheet name - 'Grid electricity (ON,CA)'.</t>
   </si>
   <si>
-    <t>CFR Data Workbook: sheet name - 'Natural gas'.</t>
-  </si>
-  <si>
     <t>CFR Data Workbook: sheet name - 'Bioethanol Portions'.</t>
   </si>
   <si>
@@ -198,6 +195,9 @@
   </si>
   <si>
     <t>p. 56-63</t>
+  </si>
+  <si>
+    <t>CFR Data Workbook: sheet name - 'Wheat (non-durum) (Global)'.</t>
   </si>
 </sst>
 </file>
@@ -2075,123 +2075,123 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{952813EB-B224-4A74-842F-0464E3E3AC57}">
   <dimension ref="A1:S154"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="47.42578125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="42.28515625" style="4" customWidth="1"/>
-    <col min="6" max="19" width="8.85546875" style="3"/>
-    <col min="20" max="16384" width="8.85546875" style="4"/>
+    <col min="1" max="1" width="4.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="47.44140625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="42.33203125" style="4" customWidth="1"/>
+    <col min="6" max="19" width="8.88671875" style="3"/>
+    <col min="20" max="16384" width="8.88671875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B2" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="51" t="s">
         <v>41</v>
-      </c>
-      <c r="C2" s="51" t="s">
-        <v>42</v>
       </c>
       <c r="D2" s="51"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" s="47" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="50" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D3" s="50"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" s="47" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="50" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D4" s="50"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" s="47" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="52" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D5" s="52"/>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="47" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D6" s="50"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" s="47" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D7" s="50"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="46" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C8" s="49"/>
       <c r="D8" s="49"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="47" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="50" t="s">
         <v>50</v>
-      </c>
-      <c r="C9" s="50" t="s">
-        <v>51</v>
       </c>
       <c r="D9" s="50"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="47" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D10" s="50"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="50" t="s">
         <v>52</v>
-      </c>
-      <c r="C11" s="50" t="s">
-        <v>53</v>
       </c>
       <c r="D11" s="50"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="2:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>0</v>
       </c>
@@ -2199,7 +2199,7 @@
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="5" t="s">
         <v>1</v>
       </c>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="F14" s="9"/>
     </row>
-    <row r="15" spans="2:6" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:6" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="10" t="s">
         <v>3</v>
       </c>
@@ -2227,7 +2227,7 @@
       <c r="E15" s="13"/>
       <c r="F15" s="14"/>
     </row>
-    <row r="16" spans="2:6" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:6" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="15" t="s">
         <v>4</v>
       </c>
@@ -2241,7 +2241,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="29.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" ht="29.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="19" t="s">
         <v>5</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="2:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="5" t="s">
         <v>10</v>
       </c>
@@ -2269,7 +2269,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="23" t="s">
         <v>0</v>
       </c>
@@ -2281,19 +2281,19 @@
       </c>
       <c r="E19" s="24"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
     </row>
-    <row r="22" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="1" t="s">
         <v>12</v>
       </c>
@@ -2301,7 +2301,7 @@
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="5" t="s">
         <v>1</v>
       </c>
@@ -2315,7 +2315,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="10" t="s">
         <v>11</v>
       </c>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="E24" s="27"/>
     </row>
-    <row r="25" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="15" t="s">
         <v>4</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="5" t="s">
         <v>10</v>
       </c>
@@ -2355,7 +2355,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27" s="23" t="s">
         <v>12</v>
       </c>
@@ -2367,19 +2367,19 @@
       </c>
       <c r="E27" s="24"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B28" s="31"/>
       <c r="C28" s="32"/>
       <c r="D28" s="33"/>
       <c r="E28" s="34"/>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="1" t="s">
         <v>13</v>
       </c>
@@ -2387,7 +2387,7 @@
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
     </row>
-    <row r="31" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="5" t="s">
         <v>1</v>
       </c>
@@ -2401,7 +2401,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="10" t="s">
         <v>14</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="23" t="s">
         <v>0</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="38" t="s">
         <v>15</v>
       </c>
@@ -2443,7 +2443,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="39" t="s">
         <v>16</v>
       </c>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="36" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="41" t="s">
         <v>17</v>
       </c>
@@ -2471,7 +2471,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="15" t="s">
         <v>12</v>
       </c>
@@ -2482,10 +2482,10 @@
         <v>19</v>
       </c>
       <c r="E37" s="30" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="38" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B38" s="5" t="s">
         <v>10</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B39" s="23" t="s">
         <v>21</v>
       </c>
@@ -2510,10 +2510,10 @@
         <v>18</v>
       </c>
       <c r="E39" s="43" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="40" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B40" s="38" t="s">
         <v>22</v>
       </c>
@@ -2524,10 +2524,10 @@
         <v>18</v>
       </c>
       <c r="E40" s="43" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="41" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B41" s="38" t="s">
         <v>23</v>
       </c>
@@ -2538,10 +2538,10 @@
         <v>18</v>
       </c>
       <c r="E41" s="43" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="42" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B42" s="38" t="s">
         <v>24</v>
       </c>
@@ -2552,10 +2552,10 @@
         <v>18</v>
       </c>
       <c r="E42" s="43" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="43" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B43" s="41" t="s">
         <v>25</v>
       </c>
@@ -2566,10 +2566,10 @@
         <v>18</v>
       </c>
       <c r="E43" s="43" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="44" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B44" s="15" t="s">
         <v>26</v>
       </c>
@@ -2580,30 +2580,30 @@
         <v>18</v>
       </c>
       <c r="E44" s="43" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
     </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
     </row>
-    <row r="47" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
     </row>
-    <row r="48" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B48" s="5" t="s">
         <v>1</v>
       </c>
@@ -2617,9 +2617,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="49" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B49" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C49" s="35">
         <v>1</v>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="E49" s="30"/>
     </row>
-    <row r="50" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B50" s="23" t="s">
         <v>4</v>
       </c>
@@ -2640,10 +2640,10 @@
         <v>9</v>
       </c>
       <c r="E50" s="30" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="51" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B51" s="5" t="s">
         <v>10</v>
       </c>
@@ -2657,9 +2657,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B52" s="23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C52" s="42">
         <v>1</v>
@@ -2669,27 +2669,27 @@
       </c>
       <c r="E52" s="43"/>
     </row>
-    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
     </row>
-    <row r="54" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
     </row>
-    <row r="55" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B55" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
     </row>
-    <row r="56" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B56" s="5" t="s">
         <v>1</v>
       </c>
@@ -2703,9 +2703,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B57" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C57" s="35">
         <v>1</v>
@@ -2715,7 +2715,7 @@
       </c>
       <c r="E57" s="30"/>
     </row>
-    <row r="58" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B58" s="5" t="s">
         <v>10</v>
       </c>
@@ -2729,9 +2729,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B59" s="23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C59" s="42">
         <v>1</v>
@@ -2741,27 +2741,27 @@
       </c>
       <c r="E59" s="43"/>
     </row>
-    <row r="60" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
       <c r="E60" s="3"/>
     </row>
-    <row r="61" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
       <c r="E61" s="3"/>
     </row>
-    <row r="62" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B62" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
       <c r="E62" s="3"/>
     </row>
-    <row r="63" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B63" s="5" t="s">
         <v>1</v>
       </c>
@@ -2775,7 +2775,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="64" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B64" s="35" t="s">
         <v>21</v>
       </c>
@@ -2787,9 +2787,9 @@
       </c>
       <c r="E64" s="30"/>
     </row>
-    <row r="65" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B65" s="23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C65" s="35">
         <v>1</v>
@@ -2799,9 +2799,9 @@
       </c>
       <c r="E65" s="45"/>
     </row>
-    <row r="66" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B66" s="35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C66" s="35">
         <v>1</v>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="E66" s="45"/>
     </row>
-    <row r="67" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B67" s="5" t="s">
         <v>10</v>
       </c>
@@ -2825,9 +2825,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B68" s="48" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C68" s="42">
         <v>1</v>
@@ -2837,26 +2837,26 @@
       </c>
       <c r="E68" s="43"/>
     </row>
-    <row r="69" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
       <c r="D69" s="3"/>
       <c r="E69" s="3"/>
     </row>
-    <row r="70" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C70" s="3"/>
       <c r="D70" s="3"/>
       <c r="E70" s="3"/>
     </row>
-    <row r="71" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B71" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C71" s="3"/>
       <c r="D71" s="3"/>
       <c r="E71" s="3"/>
     </row>
-    <row r="72" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B72" s="5" t="s">
         <v>1</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B73" s="38" t="s">
         <v>22</v>
       </c>
@@ -2882,9 +2882,9 @@
       </c>
       <c r="E73" s="30"/>
     </row>
-    <row r="74" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B74" s="23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C74" s="35">
         <v>1</v>
@@ -2894,9 +2894,9 @@
       </c>
       <c r="E74" s="45"/>
     </row>
-    <row r="75" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B75" s="35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C75" s="35">
         <v>1</v>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="E75" s="45"/>
     </row>
-    <row r="76" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B76" s="5" t="s">
         <v>10</v>
       </c>
@@ -2920,9 +2920,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="77" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B77" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C77" s="42">
         <v>1</v>
@@ -2932,463 +2932,463 @@
       </c>
       <c r="E77" s="43"/>
     </row>
-    <row r="78" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
     </row>
-    <row r="79" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
     </row>
-    <row r="80" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
     </row>
-    <row r="81" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
     </row>
-    <row r="82" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
     </row>
-    <row r="83" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
     </row>
-    <row r="84" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
     </row>
-    <row r="85" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
     </row>
-    <row r="86" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
     </row>
-    <row r="87" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
     </row>
-    <row r="88" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
     </row>
-    <row r="89" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
     </row>
-    <row r="90" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
     </row>
-    <row r="91" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
     </row>
-    <row r="93" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
     </row>
-    <row r="94" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
     </row>
-    <row r="95" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
     </row>
-    <row r="96" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
     </row>
-    <row r="97" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
     </row>
-    <row r="98" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
     </row>
-    <row r="99" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
     </row>
-    <row r="100" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
     </row>
-    <row r="101" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>
       <c r="E101" s="3"/>
     </row>
-    <row r="102" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
       <c r="D102" s="3"/>
       <c r="E102" s="3"/>
     </row>
-    <row r="103" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
       <c r="D103" s="3"/>
       <c r="E103" s="3"/>
     </row>
-    <row r="104" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
       <c r="D104" s="3"/>
       <c r="E104" s="3"/>
     </row>
-    <row r="105" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
       <c r="D105" s="3"/>
       <c r="E105" s="3"/>
     </row>
-    <row r="106" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
     </row>
-    <row r="107" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
       <c r="D107" s="3"/>
       <c r="E107" s="3"/>
     </row>
-    <row r="108" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
       <c r="E108" s="3"/>
     </row>
-    <row r="109" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
       <c r="D109" s="3"/>
       <c r="E109" s="3"/>
     </row>
-    <row r="110" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
       <c r="D110" s="3"/>
       <c r="E110" s="3"/>
     </row>
-    <row r="111" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
       <c r="D111" s="3"/>
       <c r="E111" s="3"/>
     </row>
-    <row r="112" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
       <c r="D112" s="3"/>
       <c r="E112" s="3"/>
     </row>
-    <row r="113" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
       <c r="D113" s="3"/>
       <c r="E113" s="3"/>
     </row>
-    <row r="114" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
       <c r="D114" s="3"/>
       <c r="E114" s="3"/>
     </row>
-    <row r="115" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
       <c r="D115" s="3"/>
       <c r="E115" s="3"/>
     </row>
-    <row r="116" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
       <c r="D116" s="3"/>
       <c r="E116" s="3"/>
     </row>
-    <row r="117" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
       <c r="D117" s="3"/>
       <c r="E117" s="3"/>
     </row>
-    <row r="118" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
       <c r="D118" s="3"/>
       <c r="E118" s="3"/>
     </row>
-    <row r="119" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
       <c r="D119" s="3"/>
       <c r="E119" s="3"/>
     </row>
-    <row r="120" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
       <c r="D120" s="3"/>
       <c r="E120" s="3"/>
     </row>
-    <row r="121" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
       <c r="D121" s="3"/>
       <c r="E121" s="3"/>
     </row>
-    <row r="122" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
       <c r="D122" s="3"/>
       <c r="E122" s="3"/>
     </row>
-    <row r="123" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
       <c r="D123" s="3"/>
       <c r="E123" s="3"/>
     </row>
-    <row r="124" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
       <c r="D124" s="3"/>
       <c r="E124" s="3"/>
     </row>
-    <row r="125" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
       <c r="D125" s="3"/>
       <c r="E125" s="3"/>
     </row>
-    <row r="126" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
       <c r="D126" s="3"/>
       <c r="E126" s="3"/>
     </row>
-    <row r="127" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
       <c r="D127" s="3"/>
       <c r="E127" s="3"/>
     </row>
-    <row r="128" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
       <c r="D128" s="3"/>
       <c r="E128" s="3"/>
     </row>
-    <row r="129" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
       <c r="D129" s="3"/>
       <c r="E129" s="3"/>
     </row>
-    <row r="130" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
       <c r="D130" s="3"/>
       <c r="E130" s="3"/>
     </row>
-    <row r="131" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
       <c r="D131" s="3"/>
       <c r="E131" s="3"/>
     </row>
-    <row r="132" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
       <c r="D132" s="3"/>
       <c r="E132" s="3"/>
     </row>
-    <row r="133" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
       <c r="D133" s="3"/>
       <c r="E133" s="3"/>
     </row>
-    <row r="134" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
       <c r="D134" s="3"/>
       <c r="E134" s="3"/>
     </row>
-    <row r="135" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
       <c r="D135" s="3"/>
       <c r="E135" s="3"/>
     </row>
-    <row r="136" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
       <c r="D136" s="3"/>
       <c r="E136" s="3"/>
     </row>
-    <row r="137" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B137" s="3"/>
       <c r="C137" s="3"/>
       <c r="D137" s="3"/>
       <c r="E137" s="3"/>
     </row>
-    <row r="138" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B138" s="3"/>
       <c r="C138" s="3"/>
       <c r="D138" s="3"/>
       <c r="E138" s="3"/>
     </row>
-    <row r="139" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
       <c r="D139" s="3"/>
       <c r="E139" s="3"/>
     </row>
-    <row r="140" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
       <c r="D140" s="3"/>
       <c r="E140" s="3"/>
     </row>
-    <row r="141" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
       <c r="D141" s="3"/>
       <c r="E141" s="3"/>
     </row>
-    <row r="142" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
       <c r="D142" s="3"/>
       <c r="E142" s="3"/>
     </row>
-    <row r="143" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
       <c r="D143" s="3"/>
       <c r="E143" s="3"/>
     </row>
-    <row r="144" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>
       <c r="D144" s="3"/>
       <c r="E144" s="3"/>
     </row>
-    <row r="145" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B145" s="3"/>
       <c r="C145" s="3"/>
       <c r="D145" s="3"/>
       <c r="E145" s="3"/>
     </row>
-    <row r="146" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
       <c r="D146" s="3"/>
       <c r="E146" s="3"/>
     </row>
-    <row r="147" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
       <c r="D147" s="3"/>
       <c r="E147" s="3"/>
     </row>
-    <row r="148" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
       <c r="D148" s="3"/>
       <c r="E148" s="3"/>
     </row>
-    <row r="149" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B149" s="3"/>
       <c r="C149" s="3"/>
       <c r="D149" s="3"/>
       <c r="E149" s="3"/>
     </row>
-    <row r="150" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B150" s="3"/>
       <c r="C150" s="3"/>
       <c r="D150" s="3"/>
       <c r="E150" s="3"/>
     </row>
-    <row r="151" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B151" s="3"/>
       <c r="C151" s="3"/>
       <c r="D151" s="3"/>
       <c r="E151" s="3"/>
     </row>
-    <row r="152" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B152" s="3"/>
       <c r="C152" s="3"/>
       <c r="D152" s="3"/>
       <c r="E152" s="3"/>
     </row>
-    <row r="153" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B153" s="3"/>
       <c r="C153" s="3"/>
       <c r="D153" s="3"/>
       <c r="E153" s="3"/>
     </row>
-    <row r="154" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B154" s="3"/>
       <c r="C154" s="3"/>
       <c r="D154" s="3"/>

</xml_diff>